<commit_message>
python script updated and BOM updated
</commit_message>
<xml_diff>
--- a/resources/v0.1.2/design_documents/BOM-V0.1.2.xlsx
+++ b/resources/v0.1.2/design_documents/BOM-V0.1.2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c1ed1b07ceb518fe/Documents/GitHub/core2s/resources/v0.1.2/design_documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{823F2AAE-25ED-44E6-8A76-EF5843E5E1BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06DD01CF-4235-41BE-AB0D-DE5285124C05}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{823F2AAE-25ED-44E6-8A76-EF5843E5E1BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7414D18-6417-47B6-A360-6D35DD7DCD31}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="319">
   <si>
     <t>Total Cost</t>
   </si>
@@ -981,6 +981,18 @@
   </si>
   <si>
     <t>24V AC PSU</t>
+  </si>
+  <si>
+    <t>BEING RETURNED</t>
+  </si>
+  <si>
+    <t>Honeywell Current Sensor</t>
+  </si>
+  <si>
+    <t>Honeywell CSNS300M-500 Closed Loop Sensor AC/DC Current +/- 18V, CSNS Series</t>
+  </si>
+  <si>
+    <t>Honeywell CSNS300M-500 Closed Loop Sensor AC/DC Current +/-18V, CSNS Series</t>
   </si>
 </sst>
 </file>
@@ -1095,7 +1107,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1106,6 +1118,12 @@
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1155,7 +1173,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1287,15 +1305,23 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1407,6 +1433,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4608,42 +4638,61 @@
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A117" s="13" t="s">
+      <c r="A117" s="47" t="s">
         <v>305</v>
       </c>
-      <c r="B117" s="23" t="s">
+      <c r="B117" s="48" t="s">
         <v>307</v>
       </c>
-      <c r="C117" s="10" t="s">
+      <c r="C117" s="49" t="s">
         <v>308</v>
       </c>
-      <c r="D117" s="8">
-        <v>1</v>
-      </c>
-      <c r="E117" s="8">
+      <c r="D117" s="50">
+        <v>1</v>
+      </c>
+      <c r="E117" s="50">
         <v>90.93</v>
       </c>
-      <c r="F117" s="6">
+      <c r="F117" s="51">
         <f>D117*E117</f>
         <v>90.93</v>
       </c>
-      <c r="H117" s="1" t="s">
+      <c r="G117" s="52"/>
+      <c r="H117" s="53" t="s">
         <v>306</v>
       </c>
+      <c r="I117" t="s">
+        <v>315</v>
+      </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A118" s="47"/>
-      <c r="B118" s="48"/>
-      <c r="C118" s="49"/>
-      <c r="D118" s="8"/>
-      <c r="E118" s="8"/>
-      <c r="F118" s="6"/>
-      <c r="H118" s="10"/>
+      <c r="A118" s="13" t="s">
+        <v>316</v>
+      </c>
+      <c r="B118" s="23" t="s">
+        <v>317</v>
+      </c>
+      <c r="C118" s="10">
+        <v>71240882</v>
+      </c>
+      <c r="D118" s="8">
+        <v>1</v>
+      </c>
+      <c r="E118" s="8">
+        <v>103.78</v>
+      </c>
+      <c r="F118" s="6">
+        <f>D118*E118</f>
+        <v>103.78</v>
+      </c>
+      <c r="H118" s="1" t="s">
+        <v>318</v>
+      </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A119" s="47"/>
-      <c r="B119" s="48"/>
-      <c r="C119" s="49"/>
+      <c r="A119" s="13"/>
+      <c r="B119" s="23"/>
+      <c r="C119" s="10"/>
       <c r="D119" s="8"/>
       <c r="E119" s="8"/>
       <c r="F119" s="6"/>
@@ -4699,18 +4748,18 @@
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A122" s="47"/>
-      <c r="B122" s="48"/>
-      <c r="C122" s="49"/>
+      <c r="A122" s="13"/>
+      <c r="B122" s="23"/>
+      <c r="C122" s="10"/>
       <c r="D122" s="8"/>
       <c r="E122" s="8"/>
       <c r="F122" s="6"/>
       <c r="H122" s="10"/>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A123" s="47"/>
-      <c r="B123" s="48"/>
-      <c r="C123" s="49"/>
+      <c r="A123" s="13"/>
+      <c r="B123" s="23"/>
+      <c r="C123" s="10"/>
       <c r="D123" s="8"/>
       <c r="E123" s="8"/>
       <c r="F123" s="6"/>
@@ -4735,7 +4784,7 @@
       <c r="D125" s="8"/>
       <c r="E125" s="8"/>
       <c r="F125" s="6">
-        <f t="shared" ref="F121:F127" si="5">D125*E125</f>
+        <f t="shared" ref="F125:F127" si="5">D125*E125</f>
         <v>0</v>
       </c>
       <c r="H125" s="10"/>
@@ -4880,11 +4929,12 @@
     <hyperlink ref="H117" r:id="rId111" display="https://www.digikey.com/en/products/detail/pulse-egston/N1HLR-2700MV-KA-5V/29410171?gclid=d0e0296f6f231fb67a4543cf4f2a21d9&amp;gclsrc=3p.ds&amp;msclkid=d0e0296f6f231fb67a4543cf4f2a21d9" xr:uid="{54E9C926-24F1-4758-853F-BD129F6EBDFF}"/>
     <hyperlink ref="I116" r:id="rId112" display="https://www.supplyhouse.com/Functional-Devices-TIB100A-Transformer-96VA-120-to-24-Vac-Circuit-Breaker-DIN-Rail-Mount?msockid=277021126b6a6b6a3cca367a6a576a6d" xr:uid="{0A2C36B1-5125-4F51-8575-F092A696C03C}"/>
     <hyperlink ref="H116" r:id="rId113" display="https://www.digikey.com/en/products/detail/aim-dynamics/TIB100A/28736836?msockid=277021126b6a6b6a3cca367a6a576a6d" xr:uid="{74179639-4519-4C59-BD73-C785247C9073}"/>
+    <hyperlink ref="H118" r:id="rId114" display="https://us.rs-online.com/product/honeywell/csns300m-500/71240882/" xr:uid="{D55F2F03-1317-42CE-8E65-652BDD02A6D3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId114"/>
+  <pageSetup orientation="portrait" r:id="rId115"/>
   <tableParts count="1">
-    <tablePart r:id="rId115"/>
+    <tablePart r:id="rId116"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>